<commit_message>
refactor(platform): migrar comunas/barrios/puestos de catálogos a maestras globales
- Eliminadas páginas de catálogo de campaña para comunas y barrios
- Creadas páginas maestras CRUD en /platform/maestras/ para comunas, barrios, puestos-votacion
- Agregados enlaces en sidebar de plataforma
- Queries de campaña adaptadas para filtrar por alcance territorial en vez de id_campana
- Bulk upload extendido para soportar comunas, barrios y puestos-votacion
- Eliminadas server actions y row actions de catálogo obsoletas
</commit_message>
<xml_diff>
--- a/documentos/plantilla-comunas (2).xlsx
+++ b/documentos/plantilla-comunas (2).xlsx
@@ -1,74 +1,81 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER NITRO\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB0D8D20-0C9C-4570-BAB3-B148FE156234}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="datos" sheetId="1" r:id="rId1"/>
+    <sheet name="datos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+  <si>
+    <t>municipio</t>
+  </si>
   <si>
     <t>nombre</t>
   </si>
   <si>
-    <t>COMUNA 1 CENTRO</t>
-  </si>
-  <si>
-    <t>COMUNA 2 CENTRO ORIENTAL</t>
-  </si>
-  <si>
-    <t>COMUNA 3 SUR ORIENTAL</t>
-  </si>
-  <si>
-    <t>COMUNA 4 ORIENTAL</t>
-  </si>
-  <si>
-    <t>COMUNA 5 NORORIENTAL</t>
-  </si>
-  <si>
-    <t>COMUNA 6 NORTE</t>
-  </si>
-  <si>
-    <t>COMUNA 7 NOR OCCIDENTAL</t>
-  </si>
-  <si>
-    <t>COMUNA 8 OCCIDENTAL</t>
-  </si>
-  <si>
-    <t>COMUNA 9 SUR OCCIDENTAL</t>
-  </si>
-  <si>
-    <t>COMUNA 10 SUR</t>
-  </si>
-  <si>
-    <t>NO APLICA</t>
+    <t xml:space="preserve">San José De Cúcuta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMUNA 1 CENTRO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMUNA 2 CENTRO ORIENTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMUNA 3 SUR ORIENTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMUNA 4 ORIENTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMUNA 5 NORORIENTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMUNA 6 NORTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMUNA 7 NOR OCCIDENTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMUNA 8 OCCIDENTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMUNA 9 SUR OCCIDENTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMUNA 10 SUR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NO APLICA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2">
     <font>
-      <sz val="12"/>
+      <sz val="12.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.500000"/>
+      <color indexed="64"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -81,24 +88,27 @@
   </fills>
   <borders count="1">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -110,7 +120,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -156,13 +166,13 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Thai" typeface="Angsana New"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -185,19 +195,18 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Thai" typeface="Cordia New"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -220,7 +229,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -255,16 +263,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -386,9 +398,226 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
   <a:objectDefaults>
     <a:spDef>
-      <a:spPr/>
+      <a:spPr bwMode="auto"/>
       <a:bodyPr/>
       <a:lstStyle/>
       <a:style>
@@ -407,7 +636,7 @@
       </a:style>
     </a:spDef>
     <a:lnDef>
-      <a:spPr/>
+      <a:spPr bwMode="auto"/>
       <a:bodyPr/>
       <a:lstStyle/>
       <a:style>
@@ -426,82 +655,117 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col min="1" max="1" width="26.625" bestFit="1" customWidth="1"/>
+    <col bestFit="1" min="1" max="1" width="17.875"/>
+    <col bestFit="1" customWidth="1" min="2" max="2" width="26.625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" ht="15.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="2" ht="15.75">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="3" ht="15.75">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="4" ht="15.75">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="5" ht="15.75">
+      <c r="A5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="6" ht="15.75">
+      <c r="A6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="7" ht="15.75">
+      <c r="A7" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="8" ht="15.75">
+      <c r="A8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="9" ht="15.75">
+      <c r="A9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="10" ht="15.75">
+      <c r="A10" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
         <v>11</v>
       </c>
     </row>
+    <row r="11" ht="15.75">
+      <c r="A11" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" ht="15.75">
+      <c r="A12" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1" numberStoredAsText="1"/>
-  </ignoredErrors>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>